<commit_message>
Added number of participants to ManagerSessionsData.xlsx file in Python folder
</commit_message>
<xml_diff>
--- a/Python-Fig6to7/ManagerSessionsData.xlsx
+++ b/Python-Fig6to7/ManagerSessionsData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anabelle/Documents/Quantifying Data for Extreme Low Inflow and Extreme Low Storage Storage Scenarios for Lake Mead/ImmersiveModelSessionData/ManagerSessionData-Updated-8-4-26 /"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2395274331961/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E49F069D-1497-994A-9229-97D7B8DDCBE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{E49F069D-1497-994A-9229-97D7B8DDCBE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD89FB65-B872-43B5-8326-4082D17D80FD}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{AB918D16-D3B7-EB42-8D76-4088090A27FB}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AB918D16-D3B7-EB42-8D76-4088090A27FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="28">
   <si>
     <t>Session</t>
   </si>
@@ -119,6 +119,12 @@
   </si>
   <si>
     <t>2025-10-27</t>
+  </si>
+  <si>
+    <t>Number of Participants</t>
+  </si>
+  <si>
+    <t>Total Participants</t>
   </si>
 </sst>
 </file>
@@ -141,12 +147,14 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -176,7 +184,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -389,11 +397,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -491,6 +508,24 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -827,13 +862,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5DBA0C1-1E4D-3946-A30D-FCEEAEABD221}">
-  <dimension ref="A1:G49"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:I49"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="35" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="48.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
@@ -855,8 +890,14 @@
       <c r="G1" s="25" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H1" s="38" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="41" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A2" s="34" t="s">
         <v>21</v>
       </c>
@@ -878,8 +919,15 @@
       <c r="G2" s="10">
         <v>3.9</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H2" s="37">
+        <v>3</v>
+      </c>
+      <c r="I2" s="42">
+        <f>SUM(H2:H49)</f>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A3" s="35"/>
       <c r="B3" s="1" t="s">
         <v>8</v>
@@ -902,7 +950,7 @@
         <v>0.8666666666666667</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="36"/>
       <c r="B4" s="12" t="s">
         <v>9</v>
@@ -923,7 +971,7 @@
         <v>989.5</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A5" s="34" t="s">
         <v>10</v>
       </c>
@@ -943,8 +991,11 @@
         <v>7.2</v>
       </c>
       <c r="G5" s="26"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H5" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A6" s="35"/>
       <c r="B6" s="1" t="s">
         <v>8</v>
@@ -964,7 +1015,7 @@
       </c>
       <c r="G6" s="27"/>
     </row>
-    <row r="7" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A7" s="36"/>
       <c r="B7" s="16" t="s">
         <v>9</v>
@@ -983,7 +1034,7 @@
       </c>
       <c r="G7" s="28"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A8" s="34" t="s">
         <v>22</v>
       </c>
@@ -1005,8 +1056,11 @@
       <c r="G8" s="10">
         <v>8.3000000000000007</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H8" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A9" s="35"/>
       <c r="B9" s="1" t="s">
         <v>8</v>
@@ -1029,7 +1083,7 @@
         <v>1.3174603174603177</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A10" s="36"/>
       <c r="B10" s="12" t="s">
         <v>9</v>
@@ -1050,7 +1104,7 @@
         <v>1058</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A11" s="34" t="s">
         <v>11</v>
       </c>
@@ -1072,8 +1126,11 @@
       <c r="G11" s="26">
         <v>4.4000000000000004</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H11" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A12" s="35"/>
       <c r="B12" s="1" t="s">
         <v>8</v>
@@ -1096,7 +1153,7 @@
         <v>1.375</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A13" s="36"/>
       <c r="B13" s="16" t="s">
         <v>9</v>
@@ -1117,7 +1174,7 @@
         <v>998.5</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A14" s="34" t="s">
         <v>25</v>
       </c>
@@ -1139,8 +1196,11 @@
       <c r="G14" s="21">
         <v>5.9</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H14" s="39">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A15" s="35"/>
       <c r="B15" s="1" t="s">
         <v>8</v>
@@ -1163,7 +1223,7 @@
         <v>1.3111111111111111</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A16" s="36"/>
       <c r="B16" s="12" t="s">
         <v>9</v>
@@ -1184,7 +1244,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A17" s="34" t="s">
         <v>12</v>
       </c>
@@ -1206,8 +1266,11 @@
       <c r="G17" s="10">
         <v>6.4</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H17" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A18" s="35"/>
       <c r="B18" s="1" t="s">
         <v>8</v>
@@ -1230,7 +1293,7 @@
         <v>1.0666666666666667</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A19" s="36"/>
       <c r="B19" s="12" t="s">
         <v>9</v>
@@ -1251,7 +1314,7 @@
         <v>1031</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A20" s="34" t="s">
         <v>13</v>
       </c>
@@ -1273,8 +1336,11 @@
       <c r="G20" s="10">
         <v>8</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H20" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A21" s="35"/>
       <c r="B21" s="1" t="s">
         <v>8</v>
@@ -1297,7 +1363,7 @@
         <v>1.3333333333333333</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A22" s="36"/>
       <c r="B22" s="12" t="s">
         <v>9</v>
@@ -1318,7 +1384,7 @@
         <v>1053.5</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A23" s="34" t="s">
         <v>14</v>
       </c>
@@ -1338,8 +1404,11 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="G23" s="26"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H23" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A24" s="35"/>
       <c r="B24" s="1" t="s">
         <v>8</v>
@@ -1359,7 +1428,7 @@
       </c>
       <c r="G24" s="22"/>
     </row>
-    <row r="25" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A25" s="36"/>
       <c r="B25" s="16" t="s">
         <v>9</v>
@@ -1378,7 +1447,7 @@
       </c>
       <c r="G25" s="28"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A26" s="34" t="s">
         <v>19</v>
       </c>
@@ -1398,8 +1467,11 @@
         <v>5.7</v>
       </c>
       <c r="G26" s="10"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H26" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A27" s="35"/>
       <c r="B27" s="1" t="s">
         <v>8</v>
@@ -1419,7 +1491,7 @@
       </c>
       <c r="G27" s="11"/>
     </row>
-    <row r="28" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A28" s="36"/>
       <c r="B28" s="16" t="s">
         <v>9</v>
@@ -1438,7 +1510,7 @@
       </c>
       <c r="G28" s="28"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A29" s="34" t="s">
         <v>16</v>
       </c>
@@ -1456,8 +1528,11 @@
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="10"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H29" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A30" s="35"/>
       <c r="B30" s="1" t="s">
         <v>8</v>
@@ -1474,7 +1549,7 @@
       <c r="F30" s="3"/>
       <c r="G30" s="11"/>
     </row>
-    <row r="31" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A31" s="36"/>
       <c r="B31" s="12" t="s">
         <v>9</v>
@@ -1491,7 +1566,7 @@
       <c r="F31" s="14"/>
       <c r="G31" s="15"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A32" s="34" t="s">
         <v>15</v>
       </c>
@@ -1511,8 +1586,11 @@
         <v>4.3</v>
       </c>
       <c r="G32" s="26"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H32" s="40">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A33" s="35"/>
       <c r="B33" s="1" t="s">
         <v>8</v>
@@ -1532,7 +1610,7 @@
       </c>
       <c r="G33" s="11"/>
     </row>
-    <row r="34" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A34" s="36"/>
       <c r="B34" s="12" t="s">
         <v>9</v>
@@ -1551,7 +1629,7 @@
       </c>
       <c r="G34" s="15"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A35" s="34" t="s">
         <v>20</v>
       </c>
@@ -1571,8 +1649,11 @@
         <v>3.2</v>
       </c>
       <c r="G35" s="10"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H35" s="40">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A36" s="35"/>
       <c r="B36" s="1" t="s">
         <v>8</v>
@@ -1592,7 +1673,7 @@
       </c>
       <c r="G36" s="11"/>
     </row>
-    <row r="37" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A37" s="36"/>
       <c r="B37" s="12" t="s">
         <v>9</v>
@@ -1611,7 +1692,7 @@
       </c>
       <c r="G37" s="15"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A38" s="34" t="s">
         <v>18</v>
       </c>
@@ -1629,8 +1710,11 @@
       </c>
       <c r="F38" s="7"/>
       <c r="G38" s="26"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H38" s="37">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A39" s="35"/>
       <c r="B39" s="1" t="s">
         <v>8</v>
@@ -1647,7 +1731,7 @@
       <c r="F39" s="3"/>
       <c r="G39" s="11"/>
     </row>
-    <row r="40" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A40" s="36"/>
       <c r="B40" s="16" t="s">
         <v>9</v>
@@ -1664,7 +1748,7 @@
       <c r="F40" s="18"/>
       <c r="G40" s="28"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A41" s="34" t="s">
         <v>17</v>
       </c>
@@ -1686,8 +1770,11 @@
       <c r="G41" s="10">
         <v>3.5</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H41" s="37">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A42" s="35"/>
       <c r="B42" s="1" t="s">
         <v>8</v>
@@ -1710,7 +1797,7 @@
         <v>1.09375</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A43" s="36"/>
       <c r="B43" s="12" t="s">
         <v>9</v>
@@ -1731,7 +1818,7 @@
         <v>982</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A44" s="34" t="s">
         <v>23</v>
       </c>
@@ -1751,8 +1838,11 @@
         <v>5.6</v>
       </c>
       <c r="G44" s="10"/>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H44" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A45" s="35"/>
       <c r="B45" s="1" t="s">
         <v>8</v>
@@ -1772,7 +1862,7 @@
       </c>
       <c r="G45" s="11"/>
     </row>
-    <row r="46" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A46" s="36"/>
       <c r="B46" s="12" t="s">
         <v>9</v>
@@ -1791,7 +1881,7 @@
       </c>
       <c r="G46" s="15"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A47" s="34" t="s">
         <v>24</v>
       </c>
@@ -1811,8 +1901,11 @@
         <v>3.8</v>
       </c>
       <c r="G47" s="10"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H47" s="37">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A48" s="35"/>
       <c r="B48" s="1" t="s">
         <v>8</v>
@@ -1832,7 +1925,7 @@
       </c>
       <c r="G48" s="11"/>
     </row>
-    <row r="49" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A49" s="36"/>
       <c r="B49" s="12" t="s">
         <v>9</v>
@@ -1853,22 +1946,22 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="A14:A16"/>
     <mergeCell ref="A17:A19"/>
     <mergeCell ref="A35:A37"/>
     <mergeCell ref="A44:A46"/>
     <mergeCell ref="A29:A31"/>
     <mergeCell ref="A41:A43"/>
     <mergeCell ref="A38:A40"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="A20:A22"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="A32:A34"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Duplicated correct file and replaced incorrect python file
</commit_message>
<xml_diff>
--- a/Python-Fig6to7/ManagerSessionsData.xlsx
+++ b/Python-Fig6to7/ManagerSessionsData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2395274331961/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anabelle/Documents/Quantifying Data for Extreme Low Inflow and Extreme Low Storage Storage Scenarios for Lake Mead/ImmersiveModelSessionData/ManagerSessionData-Updated-8-4-26 /"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{E49F069D-1497-994A-9229-97D7B8DDCBE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD89FB65-B872-43B5-8326-4082D17D80FD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E49F069D-1497-994A-9229-97D7B8DDCBE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AB918D16-D3B7-EB42-8D76-4088090A27FB}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{AB918D16-D3B7-EB42-8D76-4088090A27FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="26">
   <si>
     <t>Session</t>
   </si>
@@ -119,12 +119,6 @@
   </si>
   <si>
     <t>2025-10-27</t>
-  </si>
-  <si>
-    <t>Number of Participants</t>
-  </si>
-  <si>
-    <t>Total Participants</t>
   </si>
 </sst>
 </file>
@@ -147,14 +141,12 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -184,7 +176,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -397,20 +389,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -508,24 +491,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -862,13 +827,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5DBA0C1-1E4D-3946-A30D-FCEEAEABD221}">
-  <dimension ref="A1:I49"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:G49"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="48.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="35" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
@@ -890,14 +855,8 @@
       <c r="G1" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="38" t="s">
-        <v>26</v>
-      </c>
-      <c r="I1" s="41" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="34" t="s">
         <v>21</v>
       </c>
@@ -919,15 +878,8 @@
       <c r="G2" s="10">
         <v>3.9</v>
       </c>
-      <c r="H2" s="37">
-        <v>3</v>
-      </c>
-      <c r="I2" s="42">
-        <f>SUM(H2:H49)</f>
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="35"/>
       <c r="B3" s="1" t="s">
         <v>8</v>
@@ -950,7 +902,7 @@
         <v>0.8666666666666667</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="36"/>
       <c r="B4" s="12" t="s">
         <v>9</v>
@@ -971,7 +923,7 @@
         <v>989.5</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="34" t="s">
         <v>10</v>
       </c>
@@ -991,11 +943,8 @@
         <v>7.2</v>
       </c>
       <c r="G5" s="26"/>
-      <c r="H5" s="37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="35"/>
       <c r="B6" s="1" t="s">
         <v>8</v>
@@ -1015,7 +964,7 @@
       </c>
       <c r="G6" s="27"/>
     </row>
-    <row r="7" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="36"/>
       <c r="B7" s="16" t="s">
         <v>9</v>
@@ -1034,7 +983,7 @@
       </c>
       <c r="G7" s="28"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="34" t="s">
         <v>22</v>
       </c>
@@ -1056,11 +1005,8 @@
       <c r="G8" s="10">
         <v>8.3000000000000007</v>
       </c>
-      <c r="H8" s="37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.4">
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="35"/>
       <c r="B9" s="1" t="s">
         <v>8</v>
@@ -1083,7 +1029,7 @@
         <v>1.3174603174603177</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="36"/>
       <c r="B10" s="12" t="s">
         <v>9</v>
@@ -1104,7 +1050,7 @@
         <v>1058</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="34" t="s">
         <v>11</v>
       </c>
@@ -1126,11 +1072,8 @@
       <c r="G11" s="26">
         <v>4.4000000000000004</v>
       </c>
-      <c r="H11" s="37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.4">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="35"/>
       <c r="B12" s="1" t="s">
         <v>8</v>
@@ -1153,7 +1096,7 @@
         <v>1.375</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="36"/>
       <c r="B13" s="16" t="s">
         <v>9</v>
@@ -1174,7 +1117,7 @@
         <v>998.5</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="34" t="s">
         <v>25</v>
       </c>
@@ -1196,11 +1139,8 @@
       <c r="G14" s="21">
         <v>5.9</v>
       </c>
-      <c r="H14" s="39">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.4">
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="35"/>
       <c r="B15" s="1" t="s">
         <v>8</v>
@@ -1223,7 +1163,7 @@
         <v>1.3111111111111111</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="36"/>
       <c r="B16" s="12" t="s">
         <v>9</v>
@@ -1244,7 +1184,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="34" t="s">
         <v>12</v>
       </c>
@@ -1266,11 +1206,8 @@
       <c r="G17" s="10">
         <v>6.4</v>
       </c>
-      <c r="H17" s="37">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="35"/>
       <c r="B18" s="1" t="s">
         <v>8</v>
@@ -1293,7 +1230,7 @@
         <v>1.0666666666666667</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="36"/>
       <c r="B19" s="12" t="s">
         <v>9</v>
@@ -1314,7 +1251,7 @@
         <v>1031</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="34" t="s">
         <v>13</v>
       </c>
@@ -1336,11 +1273,8 @@
       <c r="G20" s="10">
         <v>8</v>
       </c>
-      <c r="H20" s="37">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="35"/>
       <c r="B21" s="1" t="s">
         <v>8</v>
@@ -1363,7 +1297,7 @@
         <v>1.3333333333333333</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="36"/>
       <c r="B22" s="12" t="s">
         <v>9</v>
@@ -1384,7 +1318,7 @@
         <v>1053.5</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="34" t="s">
         <v>14</v>
       </c>
@@ -1404,11 +1338,8 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="G23" s="26"/>
-      <c r="H23" s="37">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="35"/>
       <c r="B24" s="1" t="s">
         <v>8</v>
@@ -1428,7 +1359,7 @@
       </c>
       <c r="G24" s="22"/>
     </row>
-    <row r="25" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="36"/>
       <c r="B25" s="16" t="s">
         <v>9</v>
@@ -1447,7 +1378,7 @@
       </c>
       <c r="G25" s="28"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="34" t="s">
         <v>19</v>
       </c>
@@ -1467,11 +1398,8 @@
         <v>5.7</v>
       </c>
       <c r="G26" s="10"/>
-      <c r="H26" s="37">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="35"/>
       <c r="B27" s="1" t="s">
         <v>8</v>
@@ -1491,7 +1419,7 @@
       </c>
       <c r="G27" s="11"/>
     </row>
-    <row r="28" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="36"/>
       <c r="B28" s="16" t="s">
         <v>9</v>
@@ -1510,7 +1438,7 @@
       </c>
       <c r="G28" s="28"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="34" t="s">
         <v>16</v>
       </c>
@@ -1528,11 +1456,8 @@
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="10"/>
-      <c r="H29" s="37">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="35"/>
       <c r="B30" s="1" t="s">
         <v>8</v>
@@ -1549,7 +1474,7 @@
       <c r="F30" s="3"/>
       <c r="G30" s="11"/>
     </row>
-    <row r="31" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="36"/>
       <c r="B31" s="12" t="s">
         <v>9</v>
@@ -1566,7 +1491,7 @@
       <c r="F31" s="14"/>
       <c r="G31" s="15"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="34" t="s">
         <v>15</v>
       </c>
@@ -1586,11 +1511,8 @@
         <v>4.3</v>
       </c>
       <c r="G32" s="26"/>
-      <c r="H32" s="40">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="35"/>
       <c r="B33" s="1" t="s">
         <v>8</v>
@@ -1610,7 +1532,7 @@
       </c>
       <c r="G33" s="11"/>
     </row>
-    <row r="34" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="36"/>
       <c r="B34" s="12" t="s">
         <v>9</v>
@@ -1629,7 +1551,7 @@
       </c>
       <c r="G34" s="15"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="34" t="s">
         <v>20</v>
       </c>
@@ -1649,11 +1571,8 @@
         <v>3.2</v>
       </c>
       <c r="G35" s="10"/>
-      <c r="H35" s="40">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="35"/>
       <c r="B36" s="1" t="s">
         <v>8</v>
@@ -1673,7 +1592,7 @@
       </c>
       <c r="G36" s="11"/>
     </row>
-    <row r="37" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="36"/>
       <c r="B37" s="12" t="s">
         <v>9</v>
@@ -1692,7 +1611,7 @@
       </c>
       <c r="G37" s="15"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="34" t="s">
         <v>18</v>
       </c>
@@ -1710,11 +1629,8 @@
       </c>
       <c r="F38" s="7"/>
       <c r="G38" s="26"/>
-      <c r="H38" s="37">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="35"/>
       <c r="B39" s="1" t="s">
         <v>8</v>
@@ -1731,7 +1647,7 @@
       <c r="F39" s="3"/>
       <c r="G39" s="11"/>
     </row>
-    <row r="40" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="36"/>
       <c r="B40" s="16" t="s">
         <v>9</v>
@@ -1748,7 +1664,7 @@
       <c r="F40" s="18"/>
       <c r="G40" s="28"/>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="34" t="s">
         <v>17</v>
       </c>
@@ -1770,11 +1686,8 @@
       <c r="G41" s="10">
         <v>3.5</v>
       </c>
-      <c r="H41" s="37">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="35"/>
       <c r="B42" s="1" t="s">
         <v>8</v>
@@ -1797,7 +1710,7 @@
         <v>1.09375</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="36"/>
       <c r="B43" s="12" t="s">
         <v>9</v>
@@ -1818,7 +1731,7 @@
         <v>982</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" s="34" t="s">
         <v>23</v>
       </c>
@@ -1838,11 +1751,8 @@
         <v>5.6</v>
       </c>
       <c r="G44" s="10"/>
-      <c r="H44" s="37">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" s="35"/>
       <c r="B45" s="1" t="s">
         <v>8</v>
@@ -1862,7 +1772,7 @@
       </c>
       <c r="G45" s="11"/>
     </row>
-    <row r="46" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A46" s="36"/>
       <c r="B46" s="12" t="s">
         <v>9</v>
@@ -1881,7 +1791,7 @@
       </c>
       <c r="G46" s="15"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" s="34" t="s">
         <v>24</v>
       </c>
@@ -1901,11 +1811,8 @@
         <v>3.8</v>
       </c>
       <c r="G47" s="10"/>
-      <c r="H47" s="37">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" s="35"/>
       <c r="B48" s="1" t="s">
         <v>8</v>
@@ -1925,7 +1832,7 @@
       </c>
       <c r="G48" s="11"/>
     </row>
-    <row r="49" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A49" s="36"/>
       <c r="B49" s="12" t="s">
         <v>9</v>
@@ -1946,22 +1853,22 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="A20:A22"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="A32:A34"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="A14:A16"/>
     <mergeCell ref="A17:A19"/>
     <mergeCell ref="A35:A37"/>
     <mergeCell ref="A44:A46"/>
     <mergeCell ref="A29:A31"/>
     <mergeCell ref="A41:A43"/>
     <mergeCell ref="A38:A40"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A32:A34"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>